<commit_message>
Changed key column names + Included 3D visualisations of packing
</commit_message>
<xml_diff>
--- a/app/sample_instances/input_final.xlsx
+++ b/app/sample_instances/input_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yolina/Desktop/Optimisers/Container_packing_optimizer/app/sample_instances/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2AF59C-2DDE-E049-AAC6-AE1F6402AA9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB3AABD-720C-6F46-A4F7-0EC88FF6CEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{83FD0664-BA60-47EC-92E2-BA57C11BFD8C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17220" xr2:uid="{83FD0664-BA60-47EC-92E2-BA57C11BFD8C}"/>
   </bookViews>
   <sheets>
     <sheet name="Bestellen" sheetId="2" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="128">
   <si>
     <t>Yantian</t>
   </si>
@@ -360,9 +360,6 @@
     <t>Total number of pallets</t>
   </si>
   <si>
-    <t>External  Packaging Quantity</t>
-  </si>
-  <si>
     <t>Total pallets in row</t>
   </si>
   <si>
@@ -445,6 +442,12 @@
   </si>
   <si>
     <t>veelvoud te bestellen</t>
+  </si>
+  <si>
+    <t>Order External Packaging Quantity2</t>
+  </si>
+  <si>
+    <t>Pallet type</t>
   </si>
 </sst>
 </file>
@@ -874,10 +877,10 @@
     <tableColumn id="1" xr3:uid="{95E03F22-AA87-4443-AC5F-8858259939E1}" name="Article" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{DCDA184F-8339-4745-97BB-C47FE5DEBC7D}" name="Product name" dataDxfId="5"/>
     <tableColumn id="6" xr3:uid="{0B257032-DED7-4537-BD17-7F785641D1BE}" name="Pallet and packing size" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{0ED5C61C-AE37-4382-84D4-715706EB0DE3}" name="Pallet size" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{0ED5C61C-AE37-4382-84D4-715706EB0DE3}" name="Pallet type" dataDxfId="3"/>
     <tableColumn id="7" xr3:uid="{919CD494-A37D-478F-9F32-DC01B0AAB19A}" name="Total pallet in container" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{0D927188-4DB9-431B-B09C-99E9077B9B1F}" name="Total pallets in row" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{47E31305-A4AE-4BC4-BB61-4BAD7A10E6DB}" name="External  Packaging Quantity" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{47E31305-A4AE-4BC4-BB61-4BAD7A10E6DB}" name="Order External Packaging Quantity2" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1213,7 +1216,7 @@
     <col min="6" max="6" width="12.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.1640625" customWidth="1"/>
+    <col min="9" max="9" width="35" customWidth="1"/>
     <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -1231,30 +1234,30 @@
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B2" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B3" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C3" s="10">
         <v>6</v>
@@ -1280,7 +1283,7 @@
         <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L3">
         <f>SUM(G3:G14)</f>
@@ -1314,7 +1317,7 @@
         <v>40</v>
       </c>
       <c r="K4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L4">
         <f>(12.03-L3)*2.34*2.35</f>
@@ -1323,7 +1326,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C5" s="10">
         <v>2</v>
@@ -1348,7 +1351,7 @@
         <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L5">
         <f>(COUNT(J$17:J$1048576))-1</f>
@@ -1357,7 +1360,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B6" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C6" s="12">
         <v>6</v>
@@ -1382,7 +1385,7 @@
         <v>66</v>
       </c>
       <c r="K6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L6">
         <f>SUMPRODUCT(I:I,J:J)</f>
@@ -1391,7 +1394,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B7" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C7" s="10">
         <v>4</v>
@@ -1416,7 +1419,7 @@
         <v>44</v>
       </c>
       <c r="K7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L7">
         <f>ROUNDUP(L3/12.03,1)</f>
@@ -1425,7 +1428,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B8" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C8" s="12">
         <v>2</v>
@@ -1450,7 +1453,7 @@
         <v>22</v>
       </c>
       <c r="K8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L8">
         <f>ROUNDDOWN(R34/12.03,1)</f>
@@ -1459,7 +1462,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C9" s="10">
         <v>6</v>
@@ -1540,7 +1543,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B12" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C12" s="12">
         <v>9</v>
@@ -1567,7 +1570,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" s="10">
         <v>6</v>
@@ -1594,7 +1597,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B14" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C14" s="8">
         <v>3</v>
@@ -1626,28 +1629,28 @@
     </row>
     <row r="19" spans="2:16" ht="16" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E19" t="s">
-        <v>102</v>
-      </c>
-      <c r="F19" t="s">
         <v>101</v>
       </c>
+      <c r="F19" s="17" t="s">
+        <v>127</v>
+      </c>
       <c r="G19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I19" s="17" t="s">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>97</v>

</xml_diff>

<commit_message>
Adjusted view angle of 3d visualisations
</commit_message>
<xml_diff>
--- a/app/sample_instances/input_final.xlsx
+++ b/app/sample_instances/input_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yolina/Desktop/Optimisers/Container_packing_optimizer/app/sample_instances/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB3AABD-720C-6F46-A4F7-0EC88FF6CEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA78E7C-FACE-F948-AEDF-5A64691E7CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17220" xr2:uid="{83FD0664-BA60-47EC-92E2-BA57C11BFD8C}"/>
   </bookViews>
@@ -444,7 +444,7 @@
     <t>veelvoud te bestellen</t>
   </si>
   <si>
-    <t>Order External Packaging Quantity2</t>
+    <t>Order External Packaging Quantity</t>
   </si>
   <si>
     <t>Pallet type</t>
@@ -880,7 +880,7 @@
     <tableColumn id="4" xr3:uid="{0ED5C61C-AE37-4382-84D4-715706EB0DE3}" name="Pallet type" dataDxfId="3"/>
     <tableColumn id="7" xr3:uid="{919CD494-A37D-478F-9F32-DC01B0AAB19A}" name="Total pallet in container" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{0D927188-4DB9-431B-B09C-99E9077B9B1F}" name="Total pallets in row" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{47E31305-A4AE-4BC4-BB61-4BAD7A10E6DB}" name="Order External Packaging Quantity2" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{47E31305-A4AE-4BC4-BB61-4BAD7A10E6DB}" name="Order External Packaging Quantity" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Fixed critical issue of validator flagging but being ignored
</commit_message>
<xml_diff>
--- a/app/sample_instances/input_final.xlsx
+++ b/app/sample_instances/input_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yolina/Desktop/Optimisers/Container_packing_optimizer/app/sample_instances/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981902F4-8533-3E4C-A60F-60FBD1DD306D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EADE8D89-0F31-174E-867F-A3B6B840EDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17220" xr2:uid="{83FD0664-BA60-47EC-92E2-BA57C11BFD8C}"/>
   </bookViews>
@@ -658,6 +658,46 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -692,46 +732,6 @@
         </bottom>
         <vertical/>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </right>
-        <top style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </right>
-        <top style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </vertical>
-        <horizontal style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -892,12 +892,12 @@
     <tableColumn id="2" xr3:uid="{DCDA184F-8339-4745-97BB-C47FE5DEBC7D}" name="Product name" dataDxfId="6"/>
     <tableColumn id="6" xr3:uid="{0B257032-DED7-4537-BD17-7F785641D1BE}" name="Pallet and packing size" dataDxfId="5"/>
     <tableColumn id="4" xr3:uid="{0ED5C61C-AE37-4382-84D4-715706EB0DE3}" name="Pallet type" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{CD4E5D2C-3C97-9F48-A9E7-BFD8DB6F042E}" name="Items Ordered" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{59FDDCC4-8401-B849-B7F9-0FBA5790603D}" name="Order External Packaging Quantity" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{CD4E5D2C-3C97-9F48-A9E7-BFD8DB6F042E}" name="Items Ordered" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{59FDDCC4-8401-B849-B7F9-0FBA5790603D}" name="Order External Packaging Quantity" dataDxfId="2">
       <calculatedColumnFormula>IF(I20="","",G20/I20)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{AA526DCF-53F1-9546-9383-23BEFBDC5021}" name="Items per pallet" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{0D927188-4DB9-431B-B09C-99E9077B9B1F}" name="Total pallets in row" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{0D927188-4DB9-431B-B09C-99E9077B9B1F}" name="Total pallets in row" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Works with all 3 container sizes
</commit_message>
<xml_diff>
--- a/app/sample_instances/input_final.xlsx
+++ b/app/sample_instances/input_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yolina/Desktop/Optimisers/Container_packing_optimizer/app/sample_instances/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yolina/Desktop/Edelman_May-Sept/Contain_optimiser_May18th/Container_Optimisation-web-app/app/sample_instances/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EADE8D89-0F31-174E-867F-A3B6B840EDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDBB3768-2961-8745-927F-094EBF4178B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17220" xr2:uid="{83FD0664-BA60-47EC-92E2-BA57C11BFD8C}"/>
+    <workbookView xWindow="6220" yWindow="22360" windowWidth="26520" windowHeight="17140" xr2:uid="{83FD0664-BA60-47EC-92E2-BA57C11BFD8C}"/>
   </bookViews>
   <sheets>
     <sheet name="Bestellen" sheetId="2" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="133">
   <si>
     <t>Yantian</t>
   </si>
@@ -366,18 +366,9 @@
     <t>Pallet size</t>
   </si>
   <si>
-    <t>Pallet and packing size</t>
-  </si>
-  <si>
     <t>Product name</t>
   </si>
   <si>
-    <t>Article</t>
-  </si>
-  <si>
-    <t>Barcode</t>
-  </si>
-  <si>
     <t>D3</t>
   </si>
   <si>
@@ -441,23 +432,48 @@
     <t>veelvoud te bestellen</t>
   </si>
   <si>
-    <t>Order External Packaging Quantity</t>
-  </si>
-  <si>
-    <t>Pallet type</t>
-  </si>
-  <si>
     <t>Items per pallet</t>
   </si>
   <si>
     <t>Items Ordered</t>
+  </si>
+  <si>
+    <t>xxx</t>
+  </si>
+  <si>
+    <t>Packing</t>
+  </si>
+  <si>
+    <t>Dimensions outer / pallet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total outer / pallet </t>
+  </si>
+  <si>
+    <t>Barcode Item</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>pallet</t>
+  </si>
+  <si>
+    <t>outer carton</t>
+  </si>
+  <si>
+    <t>115x115x127cm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -488,8 +504,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -519,8 +549,20 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -627,12 +669,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -651,9 +709,21 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
@@ -887,13 +957,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DDDF6E15-7B7A-4E7B-AD16-22F32F994F7F}" name="Merge1" displayName="Merge1" ref="B19:J42" totalsRowShown="0">
   <autoFilter ref="B19:J42" xr:uid="{9539D884-44C6-4C2E-A18A-8B34BCD62477}"/>
   <tableColumns count="9">
-    <tableColumn id="3" xr3:uid="{8DD373A0-7E5C-4693-B9FC-1CE3F21B1883}" name="Barcode" dataDxfId="8"/>
-    <tableColumn id="1" xr3:uid="{95E03F22-AA87-4443-AC5F-8858259939E1}" name="Article" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{8DD373A0-7E5C-4693-B9FC-1CE3F21B1883}" name="Barcode Item" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{95E03F22-AA87-4443-AC5F-8858259939E1}" name="Item" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{DCDA184F-8339-4745-97BB-C47FE5DEBC7D}" name="Product name" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{0B257032-DED7-4537-BD17-7F785641D1BE}" name="Pallet and packing size" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{0ED5C61C-AE37-4382-84D4-715706EB0DE3}" name="Pallet type" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{0B257032-DED7-4537-BD17-7F785641D1BE}" name="Dimensions outer / pallet" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{0ED5C61C-AE37-4382-84D4-715706EB0DE3}" name="Packing" dataDxfId="4"/>
     <tableColumn id="10" xr3:uid="{CD4E5D2C-3C97-9F48-A9E7-BFD8DB6F042E}" name="Items Ordered" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{59FDDCC4-8401-B849-B7F9-0FBA5790603D}" name="Order External Packaging Quantity" dataDxfId="2">
+    <tableColumn id="11" xr3:uid="{59FDDCC4-8401-B849-B7F9-0FBA5790603D}" name="Total outer / pallet " dataDxfId="2">
       <calculatedColumnFormula>IF(I20="","",G20/I20)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{AA526DCF-53F1-9546-9383-23BEFBDC5021}" name="Items per pallet" dataDxfId="1"/>
@@ -1234,6 +1304,7 @@
   </we:alternateReferences>
   <we:properties>
     <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+    <we:property name="claude.fileId" value="&quot;8170412e-5927-4b43-9a3f-3f00ab887ef9&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -1275,57 +1346,57 @@
         <v>99</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="11" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C3" s="10">
         <v>6</v>
       </c>
-      <c r="D3" s="10" cm="1">
-        <f t="array" ref="D3:D14">SUMIFS(I$18:I$1048576,F$18:F$1048576,B$3:B$14)</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="10">
+      <c r="D3" s="10" t="e" cm="1">
+        <f t="array" ref="D3:D14">SUMIFS(I$18:I$1048576,F$19:F$1048576,B$3:B$14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E3" s="10" t="e">
         <f t="shared" ref="E3:E14" si="0">IF(D3="0","",MOD(C3-MOD(D3,C3),C3))</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F3" s="10" t="e">
         <f t="shared" ref="F3:F14" si="1">IF(D3="0","",CEILING(D3/C3,1))</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G3" s="10" t="e">
         <f>F3*'[1]Container sizes'!I25</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H3" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I25,0)*C3</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J3" t="s">
-        <v>117</v>
-      </c>
-      <c r="K3">
+        <v>114</v>
+      </c>
+      <c r="K3" t="e">
         <f>SUM(G3:G14)</f>
-        <v>11.14</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.2">
@@ -1335,61 +1406,61 @@
       <c r="C4" s="12">
         <v>4</v>
       </c>
-      <c r="D4" s="12">
-        <v>20</v>
-      </c>
-      <c r="E4" s="12">
+      <c r="D4" s="12" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E4" s="12" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F4" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F4" s="12" t="e">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="G4" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G4" s="12" t="e">
         <f>F4*'[1]Container sizes'!I25</f>
-        <v>5.75</v>
-      </c>
-      <c r="H4" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H4" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I25,0)*C4</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J4" t="s">
-        <v>116</v>
-      </c>
-      <c r="K4">
+        <v>113</v>
+      </c>
+      <c r="K4" t="e">
         <f>(12.03-K3)*2.34*2.35</f>
-        <v>4.8941099999999933</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C5" s="10">
         <v>2</v>
       </c>
-      <c r="D5" s="10">
-        <v>0</v>
-      </c>
-      <c r="E5" s="10">
+      <c r="D5" s="10" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E5" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F5" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F5" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G5" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G5" s="10" t="e">
         <f>F5*'[1]Container sizes'!I25</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H5" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I25,0)*C5</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="K5">
         <f>(COUNT(I$17:I$1048576))-1</f>
@@ -1398,32 +1469,32 @@
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B6" s="13" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C6" s="12">
         <v>6</v>
       </c>
-      <c r="D6" s="12">
-        <v>0</v>
-      </c>
-      <c r="E6" s="12">
+      <c r="D6" s="12" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E6" s="12" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F6" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F6" s="12" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G6" s="12" t="e">
         <f>F6*'[1]Container sizes'!I24</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H6" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I24,0)*C6</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="K6" t="e">
         <f>SUMPRODUCT(#REF!,I:I)</f>
@@ -1432,66 +1503,66 @@
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B7" s="11" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C7" s="10">
         <v>4</v>
       </c>
-      <c r="D7" s="10">
-        <v>0</v>
-      </c>
-      <c r="E7" s="10">
+      <c r="D7" s="10" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E7" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F7" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F7" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G7" s="10" t="e">
         <f>F7*'[1]Container sizes'!I24</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H7" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I24,0)*C7</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J7" t="s">
-        <v>110</v>
-      </c>
-      <c r="K7">
+        <v>107</v>
+      </c>
+      <c r="K7" t="e">
         <f>ROUNDUP(K3/12.03,1)</f>
-        <v>1</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" s="13" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C8" s="12">
         <v>2</v>
       </c>
-      <c r="D8" s="12">
-        <v>0</v>
-      </c>
-      <c r="E8" s="12">
+      <c r="D8" s="12" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E8" s="12" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F8" s="12" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G8" s="12" t="e">
         <f>F8*'[1]Container sizes'!I24</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H8" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I24,0)*C8</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K8">
         <f>ROUNDDOWN(S34/12.03,1)</f>
@@ -1500,29 +1571,29 @@
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C9" s="10">
         <v>6</v>
       </c>
-      <c r="D9" s="10">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10">
+      <c r="D9" s="10" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E9" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F9" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G9" s="10" t="e">
         <f>F9*'[1]Container sizes'!I23</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H9" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I23,0)*C9</f>
-        <v>6</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
@@ -1532,24 +1603,24 @@
       <c r="C10" s="12">
         <v>4</v>
       </c>
-      <c r="D10" s="12">
-        <v>20</v>
-      </c>
-      <c r="E10" s="12">
+      <c r="D10" s="12" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E10" s="12" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F10" s="12" t="e">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="G10" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G10" s="12" t="e">
         <f>F10*'[1]Container sizes'!I23</f>
-        <v>3.85</v>
-      </c>
-      <c r="H10" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H10" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I23,0)*C10</f>
-        <v>4</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
@@ -1559,105 +1630,105 @@
       <c r="C11" s="10">
         <v>2</v>
       </c>
-      <c r="D11" s="10">
-        <v>4</v>
-      </c>
-      <c r="E11" s="10">
+      <c r="D11" s="10" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E11" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F11" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="G11" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G11" s="10" t="e">
         <f>F11*'[1]Container sizes'!I23</f>
-        <v>1.54</v>
-      </c>
-      <c r="H11" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H11" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I23,0)*C11</f>
-        <v>2</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B12" s="13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C12" s="12">
         <v>9</v>
       </c>
-      <c r="D12" s="12">
-        <v>0</v>
-      </c>
-      <c r="E12" s="12">
+      <c r="D12" s="12" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E12" s="12" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F12" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F12" s="12" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G12" s="12" t="e">
         <f>F12*'[1]Container sizes'!I22</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H12" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I22,0)*C12</f>
-        <v>9</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C13" s="10">
         <v>6</v>
       </c>
-      <c r="D13" s="10">
-        <v>0</v>
-      </c>
-      <c r="E13" s="10">
+      <c r="D13" s="10" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E13" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F13" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F13" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G13" s="10" t="e">
         <f>F13*'[1]Container sizes'!I22</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H13" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I22,0)*C13</f>
-        <v>6</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B14" s="9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C14" s="8">
         <v>3</v>
       </c>
-      <c r="D14" s="8">
-        <v>0</v>
-      </c>
-      <c r="E14" s="8">
+      <c r="D14" s="8" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E14" s="8" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F14" s="8">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F14" s="8" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="8">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G14" s="8" t="e">
         <f>F14*'[1]Container sizes'!I22</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H14" s="7" t="e">
         <f>ROUNDDOWN((12.03-K3)/'[1]Container sizes'!I22,0)*C14</f>
-        <v>3</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
@@ -1665,30 +1736,39 @@
         <v>3</v>
       </c>
     </row>
+    <row r="18" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="B18" s="20"/>
+      <c r="G18" t="s">
+        <v>124</v>
+      </c>
+      <c r="I18" t="s">
+        <v>124</v>
+      </c>
+    </row>
     <row r="19" spans="2:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="B19" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C19" t="s">
-        <v>102</v>
+      <c r="B19" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>101</v>
-      </c>
-      <c r="E19" t="s">
         <v>100</v>
       </c>
-      <c r="F19" t="s">
+      <c r="E19" s="18" t="s">
         <v>126</v>
       </c>
+      <c r="F19" s="18" t="s">
+        <v>125</v>
+      </c>
       <c r="G19" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="H19" s="17" t="s">
-        <v>125</v>
+        <v>123</v>
+      </c>
+      <c r="H19" s="19" t="s">
+        <v>127</v>
       </c>
       <c r="I19" s="17" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="J19" t="s">
         <v>98</v>
@@ -1726,17 +1806,16 @@
         <v>88</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>74</v>
+        <v>132</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G20" s="2">
         <v>64</v>
       </c>
       <c r="H20" s="2">
-        <f t="shared" ref="H20:H42" si="2">IF(I20="","",G20/I20)</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I20" s="2">
         <v>4</v>
@@ -1775,13 +1854,13 @@
         <v>81</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G21" s="2">
         <v>24</v>
       </c>
       <c r="H21" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="H21:H42" si="2">IF(I21="","",G21/I21)</f>
         <v>6</v>
       </c>
       <c r="I21" s="2">
@@ -1821,7 +1900,7 @@
         <v>81</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G22" s="2">
         <v>24</v>
@@ -1867,7 +1946,7 @@
         <v>74</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G23" s="2">
         <v>32</v>
@@ -1913,7 +1992,7 @@
         <v>74</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G24" s="2">
         <v>32</v>
@@ -1959,7 +2038,7 @@
         <v>56</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="G25" s="2">
         <v>64</v>
@@ -2005,7 +2084,7 @@
         <v>60</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="G26" s="2">
         <v>4</v>
@@ -2051,7 +2130,7 @@
         <v>56</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="G27" s="2">
         <v>12</v>
@@ -2097,7 +2176,7 @@
         <v>60</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="G28" s="2">
         <v>12</v>
@@ -2143,7 +2222,7 @@
         <v>56</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="G29" s="2">
         <v>4</v>
@@ -2189,7 +2268,7 @@
         <v>51</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="G30" s="2">
         <v>0</v>
@@ -2232,7 +2311,7 @@
         <v>46</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G31" s="2">
         <v>6</v>
@@ -2274,7 +2353,7 @@
         <v>42</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G32" s="2">
         <v>6</v>
@@ -2316,7 +2395,7 @@
         <v>38</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G33" s="2">
         <v>8</v>
@@ -2358,7 +2437,7 @@
         <v>34</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G34" s="2">
         <v>9</v>
@@ -2400,7 +2479,7 @@
         <v>30</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G35" s="2">
         <v>6</v>
@@ -2442,7 +2521,7 @@
         <v>26</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G36" s="2">
         <v>7</v>
@@ -2484,7 +2563,7 @@
         <v>19</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G37" s="2">
         <v>9</v>
@@ -2526,7 +2605,7 @@
         <v>19</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G38" s="2">
         <v>9</v>
@@ -2568,7 +2647,7 @@
         <v>15</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G39" s="2">
         <v>8</v>
@@ -2610,7 +2689,7 @@
         <v>8</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G40" s="2">
         <v>6</v>
@@ -2652,7 +2731,7 @@
         <v>8</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G41" s="2">
         <v>6</v>
@@ -2694,7 +2773,7 @@
         <v>4</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="G42" s="2">
         <v>5</v>

</xml_diff>